<commit_message>
Branch: NEXT-PRE-DEVELOPMENT - feat: implement product age group filtering functionality and update product data with age group classifications
</commit_message>
<xml_diff>
--- a/store_inventory_template.xlsx
+++ b/store_inventory_template.xlsx
@@ -544,7 +544,7 @@
         <v/>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P2" t="str">
         <v/>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P3" t="str">
         <v>KIDS CYCLE</v>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P4" t="str">
         <v>KIDS CYCLE</v>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P5" t="str">
         <v>KIDS CYCLE</v>
@@ -840,7 +840,7 @@
         <v/>
       </c>
       <c r="O6" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P6" t="str">
         <v/>
@@ -852,7 +852,7 @@
         <v/>
       </c>
       <c r="S6" t="str">
-        <v xml:space="preserve">91 Alpha Cairo 24T D2TX 3.0 </v>
+        <v>91 Alpha Cairo 24T D2TX 3.0</v>
       </c>
       <c r="T6" t="str">
         <v/>
@@ -864,7 +864,7 @@
         <v>91 Alpha Cairo 24T D2TX 3.0 - KTR Cycle World</v>
       </c>
       <c r="W6" t="str">
-        <v xml:space="preserve">91 Alpha Cairo 24T D2TX 3.0 </v>
+        <v>91 Alpha Cairo 24T D2TX 3.0</v>
       </c>
       <c r="X6" t="str">
         <v>/images/products/prod_005_1.jpg</v>
@@ -914,7 +914,7 @@
         <v/>
       </c>
       <c r="O7" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P7" t="str">
         <v>NINETY ONE CYCLE</v>
@@ -988,7 +988,7 @@
         <v/>
       </c>
       <c r="O8" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P8" t="str">
         <v>LADIES CYCLE</v>
@@ -1062,7 +1062,7 @@
         <v/>
       </c>
       <c r="O9" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P9" t="str">
         <v>LADIES CYCLE</v>
@@ -1136,7 +1136,7 @@
         <v/>
       </c>
       <c r="O10" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P10" t="str">
         <v>LADIES CYCLE</v>
@@ -1210,7 +1210,7 @@
         <v/>
       </c>
       <c r="O11" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P11" t="str">
         <v>avon gear cycle, avon cycle</v>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
       <c r="O12" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P12" t="str">
         <v>KIDS CYCLE</v>
@@ -1358,7 +1358,7 @@
         <v/>
       </c>
       <c r="O13" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P13" t="str">
         <v>LADIES CYCLE</v>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
       <c r="O14" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P14" t="str">
         <v>AVON CYCLES, FAT CYCLES</v>
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="O15" t="str">
-        <v/>
+        <v>2-5 Years</v>
       </c>
       <c r="P15" t="str">
         <v>KIDS CYCLE</v>
@@ -1580,7 +1580,7 @@
         <v/>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>2-5 Years</v>
       </c>
       <c r="P16" t="str">
         <v>KIDS CYCLE</v>
@@ -1654,7 +1654,7 @@
         <v/>
       </c>
       <c r="O17" t="str">
-        <v/>
+        <v>5-8 Years</v>
       </c>
       <c r="P17" t="str">
         <v>KIDS CYCLE</v>
@@ -1728,7 +1728,7 @@
         <v/>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P18" t="str">
         <v>KIDS CYCLE</v>
@@ -1802,7 +1802,7 @@
         <v/>
       </c>
       <c r="O19" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P19" t="str">
         <v>KIDS CYCLE</v>
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P20" t="str">
         <v>hercules cycle</v>
@@ -1950,7 +1950,7 @@
         <v/>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P21" t="str">
         <v>mtb cycles</v>
@@ -2024,7 +2024,7 @@
         <v/>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P22" t="str">
         <v>ELECTRIC</v>
@@ -2098,7 +2098,7 @@
         <v/>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P23" t="str">
         <v>ELECTRIC</v>
@@ -2172,7 +2172,7 @@
         <v/>
       </c>
       <c r="O24" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P24" t="str">
         <v/>
@@ -2246,7 +2246,7 @@
         <v/>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P25" t="str">
         <v>raleigh cycle</v>
@@ -2320,7 +2320,7 @@
         <v/>
       </c>
       <c r="O26" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P26" t="str">
         <v>ELECTRIC</v>
@@ -2394,7 +2394,7 @@
         <v>BLACK WITH SEA GREEN</v>
       </c>
       <c r="O27" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P27" t="str">
         <v/>
@@ -2468,7 +2468,7 @@
         <v/>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P28" t="str">
         <v>TORONTO CYCLES, KTR CYCLE WORLD</v>
@@ -2542,7 +2542,7 @@
         <v/>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P29" t="str">
         <v>GEAR CYCLE</v>
@@ -2616,7 +2616,7 @@
         <v/>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P30" t="str">
         <v>ELECTRIC</v>
@@ -2690,7 +2690,7 @@
         <v/>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P31" t="str">
         <v>KIDS CYCLE</v>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="O32" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P32" t="str">
         <v>KIDS CYCLE</v>
@@ -2838,7 +2838,7 @@
         <v/>
       </c>
       <c r="O33" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P33" t="str">
         <v>ELECTRIC</v>
@@ -2912,7 +2912,7 @@
         <v/>
       </c>
       <c r="O34" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P34" t="str">
         <v>GEAR</v>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
       <c r="O35" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P35" t="str">
         <v>ADULT</v>
@@ -3060,7 +3060,7 @@
         <v/>
       </c>
       <c r="O36" t="str">
-        <v/>
+        <v>2-5 Years</v>
       </c>
       <c r="P36" t="str">
         <v>KIDS CYCLE</v>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="O37" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P37" t="str">
         <v>KIDS CYCLE</v>
@@ -3208,7 +3208,7 @@
         <v/>
       </c>
       <c r="O38" t="str">
-        <v/>
+        <v>5-8 Years</v>
       </c>
       <c r="P38" t="str">
         <v>KIDS CYCLE</v>
@@ -3282,7 +3282,7 @@
         <v/>
       </c>
       <c r="O39" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P39" t="str">
         <v>ADULT</v>
@@ -3356,7 +3356,7 @@
         <v/>
       </c>
       <c r="O40" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P40" t="str">
         <v>ADULT</v>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
       <c r="S40" t="str">
-        <v xml:space="preserve">Hercules Rift IC FX DD 24T </v>
+        <v>Hercules Rift IC FX DD 24T</v>
       </c>
       <c r="T40" t="str">
         <v/>
@@ -3380,7 +3380,7 @@
         <v>Hercules Rift IC FX DD 24T - KTR Cycle World</v>
       </c>
       <c r="W40" t="str">
-        <v xml:space="preserve">Hercules Rift IC FX DD 24T </v>
+        <v>Hercules Rift IC FX DD 24T</v>
       </c>
       <c r="X40" t="str">
         <v>/images/products/prod_039_1.jpg</v>
@@ -3430,7 +3430,7 @@
         <v/>
       </c>
       <c r="O41" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P41" t="str">
         <v>ADULT</v>
@@ -3442,7 +3442,7 @@
         <v/>
       </c>
       <c r="S41" t="str">
-        <v xml:space="preserve">Hercules Rift IC FX DD 26T </v>
+        <v>Hercules Rift IC FX DD 26T</v>
       </c>
       <c r="T41" t="str">
         <v/>
@@ -3454,7 +3454,7 @@
         <v>Hercules Rift IC FX DD 26T - KTR Cycle World</v>
       </c>
       <c r="W41" t="str">
-        <v xml:space="preserve">Hercules Rift IC FX DD 26T </v>
+        <v>Hercules Rift IC FX DD 26T</v>
       </c>
       <c r="X41" t="str">
         <v>/images/products/prod_040_1.jpg</v>
@@ -3504,7 +3504,7 @@
         <v/>
       </c>
       <c r="O42" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P42" t="str">
         <v>ADULT</v>
@@ -3516,7 +3516,7 @@
         <v/>
       </c>
       <c r="S42" t="str">
-        <v xml:space="preserve">Hercules Rift IC RF VB 24T </v>
+        <v>Hercules Rift IC RF VB 24T</v>
       </c>
       <c r="T42" t="str">
         <v/>
@@ -3528,7 +3528,7 @@
         <v>Hercules Rift IC RF VB 24T - KTR Cycle World</v>
       </c>
       <c r="W42" t="str">
-        <v xml:space="preserve">Hercules Rift IC RF VB 24T </v>
+        <v>Hercules Rift IC RF VB 24T</v>
       </c>
       <c r="X42" t="str">
         <v>/images/products/prod_041_1.jpg</v>
@@ -3578,7 +3578,7 @@
         <v/>
       </c>
       <c r="O43" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P43" t="str">
         <v>ADULT</v>
@@ -3652,7 +3652,7 @@
         <v/>
       </c>
       <c r="O44" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P44" t="str">
         <v>ELECTRIC</v>
@@ -3726,7 +3726,7 @@
         <v/>
       </c>
       <c r="O45" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P45" t="str">
         <v>ELECTRIC</v>
@@ -3800,7 +3800,7 @@
         <v/>
       </c>
       <c r="O46" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P46" t="str">
         <v>ELECTRIC</v>
@@ -3874,7 +3874,7 @@
         <v/>
       </c>
       <c r="O47" t="str">
-        <v/>
+        <v>8-12 Years</v>
       </c>
       <c r="P47" t="str">
         <v>KIDS CYCLE</v>
@@ -3948,7 +3948,7 @@
         <v/>
       </c>
       <c r="O48" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P48" t="str">
         <v>LADIES CYCLE</v>
@@ -4022,7 +4022,7 @@
         <v/>
       </c>
       <c r="O49" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P49" t="str">
         <v>ADULT</v>
@@ -4034,7 +4034,7 @@
         <v/>
       </c>
       <c r="S49" t="str">
-        <v xml:space="preserve">HURRICANE 26T </v>
+        <v>HURRICANE 26T</v>
       </c>
       <c r="T49" t="str">
         <v/>
@@ -4046,7 +4046,7 @@
         <v>HURRICANE 26T - KTR Cycle World</v>
       </c>
       <c r="W49" t="str">
-        <v xml:space="preserve">HURRICANE 26T </v>
+        <v>HURRICANE 26T</v>
       </c>
       <c r="X49" t="str">
         <v>/images/products/prod_048_1.jpg</v>
@@ -4096,7 +4096,7 @@
         <v/>
       </c>
       <c r="O50" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P50" t="str">
         <v>ADULT</v>
@@ -4170,7 +4170,7 @@
         <v/>
       </c>
       <c r="O51" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P51" t="str">
         <v>ADULT</v>
@@ -4244,7 +4244,7 @@
         <v/>
       </c>
       <c r="O52" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P52" t="str">
         <v>KIDS CYCLE</v>
@@ -4318,7 +4318,7 @@
         <v/>
       </c>
       <c r="O53" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P53" t="str">
         <v>GEAR</v>
@@ -4392,7 +4392,7 @@
         <v/>
       </c>
       <c r="O54" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P54" t="str">
         <v>GEAR</v>
@@ -4466,7 +4466,7 @@
         <v/>
       </c>
       <c r="O55" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P55" t="str">
         <v>GEAR</v>
@@ -4540,7 +4540,7 @@
         <v/>
       </c>
       <c r="O56" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P56" t="str">
         <v>AOKI,ELECTRIC</v>
@@ -4614,7 +4614,7 @@
         <v/>
       </c>
       <c r="O57" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P57" t="str">
         <v>ADULT</v>
@@ -4626,7 +4626,7 @@
         <v/>
       </c>
       <c r="S57" t="str">
-        <v xml:space="preserve">NAVARRO ONE </v>
+        <v>NAVARRO ONE</v>
       </c>
       <c r="T57" t="str">
         <v/>
@@ -4638,7 +4638,7 @@
         <v>NAVARRO ONE - KTR Cycle World</v>
       </c>
       <c r="W57" t="str">
-        <v xml:space="preserve">NAVARRO ONE </v>
+        <v>NAVARRO ONE</v>
       </c>
       <c r="X57" t="str">
         <v>/images/products/prod_056_1.jpg,/images/products/prod_056_2.jpg</v>
@@ -4688,7 +4688,7 @@
         <v/>
       </c>
       <c r="O58" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P58" t="str">
         <v>ADULT</v>
@@ -4762,7 +4762,7 @@
         <v/>
       </c>
       <c r="O59" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P59" t="str">
         <v>ADULT</v>
@@ -4836,7 +4836,7 @@
         <v/>
       </c>
       <c r="O60" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P60" t="str">
         <v>ADULT</v>
@@ -4910,7 +4910,7 @@
         <v/>
       </c>
       <c r="O61" t="str">
-        <v/>
+        <v>12-15 Years</v>
       </c>
       <c r="P61" t="str">
         <v>ADULT</v>
@@ -4984,7 +4984,7 @@
         <v/>
       </c>
       <c r="O62" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P62" t="str">
         <v>ADULT</v>
@@ -5058,7 +5058,7 @@
         <v/>
       </c>
       <c r="O63" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P63" t="str">
         <v>ADULT</v>
@@ -5132,7 +5132,7 @@
         <v/>
       </c>
       <c r="O64" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P64" t="str">
         <v>ADULT</v>
@@ -5206,7 +5206,7 @@
         <v/>
       </c>
       <c r="O65" t="str">
-        <v/>
+        <v>15+ Years</v>
       </c>
       <c r="P65" t="str">
         <v>AOKI,ELECTRIC</v>

</xml_diff>